<commit_message>
Edit README and Add docker files
</commit_message>
<xml_diff>
--- a/tasks/Journal_sanquer_wilstan.xlsx
+++ b/tasks/Journal_sanquer_wilstan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilstan.sanquer\Desktop\Github\SquidTchat\tasks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{79C17628-01F1-4CEA-A62C-F5382CB4F915}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93DC0713-1F2D-4EE8-81F3-587B97F82264}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{80F6D908-82BF-40D3-B5DB-CACD124443E4}"/>
   </bookViews>
@@ -35,9 +35,63 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
+  <si>
+    <t>Journal d’activité – Projet SquidTchat – Sanquer Wilstan</t>
+  </si>
+  <si>
+    <t>Jour</t>
+  </si>
+  <si>
+    <t>Nombre total d’heures travaillées</t>
+  </si>
+  <si>
+    <t>Détails des tâches effectuées</t>
+  </si>
+  <si>
+    <t>4H</t>
+  </si>
+  <si>
+    <t>1H</t>
+  </si>
+  <si>
+    <t>Séances</t>
+  </si>
+  <si>
+    <t>Séances 1</t>
+  </si>
+  <si>
+    <t>Séances 2</t>
+  </si>
+  <si>
+    <t>Séances 3</t>
+  </si>
+  <si>
+    <t>Séances 4</t>
+  </si>
+  <si>
+    <t>Séances 5</t>
+  </si>
+  <si>
+    <t>Séances 6</t>
+  </si>
+  <si>
+    <t>Séances 7</t>
+  </si>
+  <si>
+    <t>Rédaction du cahier des charges, réalisation des diagrammes de cas d'utilisation, conception des maquettes d'interface 
+et initialisation du dépôt GitHub avec l'équipe.</t>
+  </si>
+  <si>
+    <t>Création de l'arborescence des dossiers du projet et mise à jour corrective du cahier des charges suite aux premiers retours du professeur.</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -45,16 +99,42 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="16"/>
+      <color theme="0" tint="-4.9989318521683403E-2"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -62,12 +142,170 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -402,9 +640,567 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EF07D86-D2F8-4F32-A268-7E13E7D471B5}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:R26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A1" s="20" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+      <c r="L1" s="20"/>
+      <c r="M1" s="20"/>
+      <c r="N1" s="20"/>
+      <c r="O1" s="20"/>
+      <c r="P1" s="20"/>
+      <c r="Q1" s="20"/>
+      <c r="R1" s="20"/>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A2" s="20"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="20"/>
+      <c r="L2" s="20"/>
+      <c r="M2" s="20"/>
+      <c r="N2" s="20"/>
+      <c r="O2" s="20"/>
+      <c r="P2" s="20"/>
+      <c r="Q2" s="20"/>
+      <c r="R2" s="20"/>
+    </row>
+    <row r="3" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="21"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="21" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H3" s="4"/>
+      <c r="I3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
+      <c r="P3" s="3"/>
+      <c r="Q3" s="3"/>
+      <c r="R3" s="4"/>
+    </row>
+    <row r="4" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="21"/>
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="6"/>
+      <c r="K4" s="6"/>
+      <c r="L4" s="6"/>
+      <c r="M4" s="6"/>
+      <c r="N4" s="6"/>
+      <c r="O4" s="6"/>
+      <c r="P4" s="6"/>
+      <c r="Q4" s="6"/>
+      <c r="R4" s="7"/>
+    </row>
+    <row r="5" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="21"/>
+      <c r="B5" s="21"/>
+      <c r="C5" s="21"/>
+      <c r="D5" s="21"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="7"/>
+      <c r="I5" s="5"/>
+      <c r="J5" s="6"/>
+      <c r="K5" s="6"/>
+      <c r="L5" s="6"/>
+      <c r="M5" s="6"/>
+      <c r="N5" s="6"/>
+      <c r="O5" s="6"/>
+      <c r="P5" s="6"/>
+      <c r="Q5" s="6"/>
+      <c r="R5" s="7"/>
+    </row>
+    <row r="6" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="21"/>
+      <c r="B6" s="21"/>
+      <c r="C6" s="21"/>
+      <c r="D6" s="21"/>
+      <c r="E6" s="21"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="7"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="6"/>
+      <c r="K6" s="6"/>
+      <c r="L6" s="6"/>
+      <c r="M6" s="6"/>
+      <c r="N6" s="6"/>
+      <c r="O6" s="6"/>
+      <c r="P6" s="6"/>
+      <c r="Q6" s="6"/>
+      <c r="R6" s="7"/>
+    </row>
+    <row r="7" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="21"/>
+      <c r="B7" s="21"/>
+      <c r="C7" s="21"/>
+      <c r="D7" s="21"/>
+      <c r="E7" s="21"/>
+      <c r="F7" s="21"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="5"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="7"/>
+    </row>
+    <row r="8" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="21"/>
+      <c r="B8" s="21"/>
+      <c r="C8" s="21"/>
+      <c r="D8" s="21"/>
+      <c r="E8" s="21"/>
+      <c r="F8" s="21"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="9"/>
+      <c r="K8" s="9"/>
+      <c r="L8" s="9"/>
+      <c r="M8" s="9"/>
+      <c r="N8" s="9"/>
+      <c r="O8" s="9"/>
+      <c r="P8" s="9"/>
+      <c r="Q8" s="9"/>
+      <c r="R8" s="10"/>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A9" s="19">
+        <v>46094</v>
+      </c>
+      <c r="B9" s="18"/>
+      <c r="C9" s="18"/>
+      <c r="D9" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="H9" s="13"/>
+      <c r="I9" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="J9" s="12"/>
+      <c r="K9" s="12"/>
+      <c r="L9" s="12"/>
+      <c r="M9" s="12"/>
+      <c r="N9" s="12"/>
+      <c r="O9" s="12"/>
+      <c r="P9" s="12"/>
+      <c r="Q9" s="12"/>
+      <c r="R9" s="13"/>
+    </row>
+    <row r="10" spans="1:18" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="18"/>
+      <c r="B10" s="18"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
+      <c r="G10" s="14"/>
+      <c r="H10" s="16"/>
+      <c r="I10" s="14"/>
+      <c r="J10" s="15"/>
+      <c r="K10" s="15"/>
+      <c r="L10" s="15"/>
+      <c r="M10" s="15"/>
+      <c r="N10" s="15"/>
+      <c r="O10" s="15"/>
+      <c r="P10" s="15"/>
+      <c r="Q10" s="15"/>
+      <c r="R10" s="16"/>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A11" s="19">
+        <v>46098</v>
+      </c>
+      <c r="B11" s="18"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="E11" s="18"/>
+      <c r="F11" s="18"/>
+      <c r="G11" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="H11" s="13"/>
+      <c r="I11" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="J11" s="12"/>
+      <c r="K11" s="12"/>
+      <c r="L11" s="12"/>
+      <c r="M11" s="12"/>
+      <c r="N11" s="12"/>
+      <c r="O11" s="12"/>
+      <c r="P11" s="12"/>
+      <c r="Q11" s="12"/>
+      <c r="R11" s="13"/>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A12" s="18"/>
+      <c r="B12" s="18"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="18"/>
+      <c r="F12" s="18"/>
+      <c r="G12" s="14"/>
+      <c r="H12" s="16"/>
+      <c r="I12" s="14"/>
+      <c r="J12" s="15"/>
+      <c r="K12" s="15"/>
+      <c r="L12" s="15"/>
+      <c r="M12" s="15"/>
+      <c r="N12" s="15"/>
+      <c r="O12" s="15"/>
+      <c r="P12" s="15"/>
+      <c r="Q12" s="15"/>
+      <c r="R12" s="16"/>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A13" s="19">
+        <v>46104</v>
+      </c>
+      <c r="B13" s="18"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="E13" s="18"/>
+      <c r="F13" s="18"/>
+      <c r="G13" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="H13" s="13"/>
+      <c r="I13" s="17"/>
+      <c r="J13" s="12"/>
+      <c r="K13" s="12"/>
+      <c r="L13" s="12"/>
+      <c r="M13" s="12"/>
+      <c r="N13" s="12"/>
+      <c r="O13" s="12"/>
+      <c r="P13" s="12"/>
+      <c r="Q13" s="12"/>
+      <c r="R13" s="13"/>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A14" s="18"/>
+      <c r="B14" s="18"/>
+      <c r="C14" s="18"/>
+      <c r="D14" s="18"/>
+      <c r="E14" s="18"/>
+      <c r="F14" s="18"/>
+      <c r="G14" s="14"/>
+      <c r="H14" s="16"/>
+      <c r="I14" s="14"/>
+      <c r="J14" s="15"/>
+      <c r="K14" s="15"/>
+      <c r="L14" s="15"/>
+      <c r="M14" s="15"/>
+      <c r="N14" s="15"/>
+      <c r="O14" s="15"/>
+      <c r="P14" s="15"/>
+      <c r="Q14" s="15"/>
+      <c r="R14" s="16"/>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A15" s="18"/>
+      <c r="B15" s="18"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="18"/>
+      <c r="F15" s="18"/>
+      <c r="G15" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="H15" s="13"/>
+      <c r="I15" s="17"/>
+      <c r="J15" s="12"/>
+      <c r="K15" s="12"/>
+      <c r="L15" s="12"/>
+      <c r="M15" s="12"/>
+      <c r="N15" s="12"/>
+      <c r="O15" s="12"/>
+      <c r="P15" s="12"/>
+      <c r="Q15" s="12"/>
+      <c r="R15" s="13"/>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A16" s="18"/>
+      <c r="B16" s="18"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="18"/>
+      <c r="E16" s="18"/>
+      <c r="F16" s="18"/>
+      <c r="G16" s="14"/>
+      <c r="H16" s="16"/>
+      <c r="I16" s="14"/>
+      <c r="J16" s="15"/>
+      <c r="K16" s="15"/>
+      <c r="L16" s="15"/>
+      <c r="M16" s="15"/>
+      <c r="N16" s="15"/>
+      <c r="O16" s="15"/>
+      <c r="P16" s="15"/>
+      <c r="Q16" s="15"/>
+      <c r="R16" s="16"/>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A17" s="18"/>
+      <c r="B17" s="18"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="18"/>
+      <c r="E17" s="18"/>
+      <c r="F17" s="18"/>
+      <c r="G17" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="H17" s="13"/>
+      <c r="I17" s="17"/>
+      <c r="J17" s="12"/>
+      <c r="K17" s="12"/>
+      <c r="L17" s="12"/>
+      <c r="M17" s="12"/>
+      <c r="N17" s="12"/>
+      <c r="O17" s="12"/>
+      <c r="P17" s="12"/>
+      <c r="Q17" s="12"/>
+      <c r="R17" s="13"/>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A18" s="18"/>
+      <c r="B18" s="18"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="18"/>
+      <c r="E18" s="18"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="14"/>
+      <c r="H18" s="16"/>
+      <c r="I18" s="14"/>
+      <c r="J18" s="15"/>
+      <c r="K18" s="15"/>
+      <c r="L18" s="15"/>
+      <c r="M18" s="15"/>
+      <c r="N18" s="15"/>
+      <c r="O18" s="15"/>
+      <c r="P18" s="15"/>
+      <c r="Q18" s="15"/>
+      <c r="R18" s="16"/>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A19" s="18"/>
+      <c r="B19" s="18"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="18"/>
+      <c r="E19" s="18"/>
+      <c r="F19" s="18"/>
+      <c r="G19" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="H19" s="13"/>
+      <c r="I19" s="17"/>
+      <c r="J19" s="12"/>
+      <c r="K19" s="12"/>
+      <c r="L19" s="12"/>
+      <c r="M19" s="12"/>
+      <c r="N19" s="12"/>
+      <c r="O19" s="12"/>
+      <c r="P19" s="12"/>
+      <c r="Q19" s="12"/>
+      <c r="R19" s="13"/>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A20" s="18"/>
+      <c r="B20" s="18"/>
+      <c r="C20" s="18"/>
+      <c r="D20" s="18"/>
+      <c r="E20" s="18"/>
+      <c r="F20" s="18"/>
+      <c r="G20" s="14"/>
+      <c r="H20" s="16"/>
+      <c r="I20" s="14"/>
+      <c r="J20" s="15"/>
+      <c r="K20" s="15"/>
+      <c r="L20" s="15"/>
+      <c r="M20" s="15"/>
+      <c r="N20" s="15"/>
+      <c r="O20" s="15"/>
+      <c r="P20" s="15"/>
+      <c r="Q20" s="15"/>
+      <c r="R20" s="16"/>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A21" s="18"/>
+      <c r="B21" s="18"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="18"/>
+      <c r="E21" s="18"/>
+      <c r="F21" s="18"/>
+      <c r="G21" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="H21" s="18"/>
+      <c r="I21" s="18"/>
+      <c r="J21" s="18"/>
+      <c r="K21" s="18"/>
+      <c r="L21" s="18"/>
+      <c r="M21" s="18"/>
+      <c r="N21" s="18"/>
+      <c r="O21" s="18"/>
+      <c r="P21" s="18"/>
+      <c r="Q21" s="18"/>
+      <c r="R21" s="18"/>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A22" s="18"/>
+      <c r="B22" s="18"/>
+      <c r="C22" s="18"/>
+      <c r="D22" s="18"/>
+      <c r="E22" s="18"/>
+      <c r="F22" s="18"/>
+      <c r="G22" s="18"/>
+      <c r="H22" s="18"/>
+      <c r="I22" s="18"/>
+      <c r="J22" s="18"/>
+      <c r="K22" s="18"/>
+      <c r="L22" s="18"/>
+      <c r="M22" s="18"/>
+      <c r="N22" s="18"/>
+      <c r="O22" s="18"/>
+      <c r="P22" s="18"/>
+      <c r="Q22" s="18"/>
+      <c r="R22" s="18"/>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A23" s="1"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
+      <c r="G23" s="1"/>
+      <c r="H23" s="1"/>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A24" s="1"/>
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+      <c r="F24" s="1"/>
+      <c r="G24" s="1"/>
+      <c r="H24" s="1"/>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A25" s="1"/>
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+      <c r="F25" s="1"/>
+      <c r="G25" s="1"/>
+      <c r="H25" s="1"/>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A26" s="1"/>
+      <c r="B26" s="1"/>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="1"/>
+      <c r="H26" s="1"/>
+    </row>
+  </sheetData>
+  <mergeCells count="33">
+    <mergeCell ref="A1:R2"/>
+    <mergeCell ref="A3:C8"/>
+    <mergeCell ref="D3:F8"/>
+    <mergeCell ref="D21:F22"/>
+    <mergeCell ref="A19:C20"/>
+    <mergeCell ref="A21:C22"/>
+    <mergeCell ref="D9:F10"/>
+    <mergeCell ref="D11:F12"/>
+    <mergeCell ref="D13:F14"/>
+    <mergeCell ref="D15:F16"/>
+    <mergeCell ref="D17:F18"/>
+    <mergeCell ref="D19:F20"/>
+    <mergeCell ref="A9:C10"/>
+    <mergeCell ref="A11:C12"/>
+    <mergeCell ref="A13:C14"/>
+    <mergeCell ref="A15:C16"/>
+    <mergeCell ref="A17:C18"/>
+    <mergeCell ref="I17:R18"/>
+    <mergeCell ref="I19:R20"/>
+    <mergeCell ref="I21:R22"/>
+    <mergeCell ref="G3:H8"/>
+    <mergeCell ref="G9:H10"/>
+    <mergeCell ref="G11:H12"/>
+    <mergeCell ref="G15:H16"/>
+    <mergeCell ref="G13:H14"/>
+    <mergeCell ref="G17:H18"/>
+    <mergeCell ref="G19:H20"/>
+    <mergeCell ref="G21:H22"/>
+    <mergeCell ref="I3:R8"/>
+    <mergeCell ref="I9:R10"/>
+    <mergeCell ref="I11:R12"/>
+    <mergeCell ref="I13:R14"/>
+    <mergeCell ref="I15:R16"/>
+  </mergeCells>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add CSS pages index, forum
</commit_message>
<xml_diff>
--- a/tasks/Journal_sanquer_wilstan.xlsx
+++ b/tasks/Journal_sanquer_wilstan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilstan.sanquer\Desktop\Github\SquidTchat\tasks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B5718D3-043C-4C56-896C-ED3E2243ED33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4F70131-754C-420F-84E8-FF835728A916}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{80F6D908-82BF-40D3-B5DB-CACD124443E4}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
   <si>
     <t>Journal d’activité – Projet SquidTchat – Sanquer Wilstan</t>
   </si>
@@ -97,6 +97,12 @@
   </si>
   <si>
     <t>Création des pages HTML, des feuilles de style CSS et initialisation de la communication WebSocket entre le client et le serveur.</t>
+  </si>
+  <si>
+    <t>2H</t>
+  </si>
+  <si>
+    <t>Application des feuilles de style CSS aux pages index.html et forum.html, et création du fichier JavaScript pour l'initialisation de la logique du chat.</t>
   </si>
 </sst>
 </file>
@@ -253,36 +259,36 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -315,13 +321,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -662,58 +665,58 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
-      <c r="P1" s="1"/>
-      <c r="Q1" s="1"/>
-      <c r="R1" s="1"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="21"/>
+      <c r="L1" s="21"/>
+      <c r="M1" s="21"/>
+      <c r="N1" s="21"/>
+      <c r="O1" s="21"/>
+      <c r="P1" s="21"/>
+      <c r="Q1" s="21"/>
+      <c r="R1" s="21"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
-      <c r="N2" s="1"/>
-      <c r="O2" s="1"/>
-      <c r="P2" s="1"/>
-      <c r="Q2" s="1"/>
-      <c r="R2" s="1"/>
+      <c r="A2" s="21"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
+      <c r="I2" s="21"/>
+      <c r="J2" s="21"/>
+      <c r="K2" s="21"/>
+      <c r="L2" s="21"/>
+      <c r="M2" s="21"/>
+      <c r="N2" s="21"/>
+      <c r="O2" s="21"/>
+      <c r="P2" s="21"/>
+      <c r="Q2" s="21"/>
+      <c r="R2" s="21"/>
     </row>
     <row r="3" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2" t="s">
+      <c r="B3" s="22"/>
+      <c r="C3" s="22"/>
+      <c r="D3" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
+      <c r="E3" s="22"/>
+      <c r="F3" s="22"/>
       <c r="G3" s="11" t="s">
         <v>6</v>
       </c>
@@ -732,12 +735,12 @@
       <c r="R3" s="12"/>
     </row>
     <row r="4" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
+      <c r="A4" s="22"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
       <c r="G4" s="13"/>
       <c r="H4" s="14"/>
       <c r="I4" s="13"/>
@@ -752,12 +755,12 @@
       <c r="R4" s="14"/>
     </row>
     <row r="5" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
+      <c r="A5" s="22"/>
+      <c r="B5" s="22"/>
+      <c r="C5" s="22"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="22"/>
       <c r="G5" s="13"/>
       <c r="H5" s="14"/>
       <c r="I5" s="13"/>
@@ -772,12 +775,12 @@
       <c r="R5" s="14"/>
     </row>
     <row r="6" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
+      <c r="A6" s="22"/>
+      <c r="B6" s="22"/>
+      <c r="C6" s="22"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="22"/>
+      <c r="F6" s="22"/>
       <c r="G6" s="13"/>
       <c r="H6" s="14"/>
       <c r="I6" s="13"/>
@@ -792,12 +795,12 @@
       <c r="R6" s="14"/>
     </row>
     <row r="7" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
+      <c r="A7" s="22"/>
+      <c r="B7" s="22"/>
+      <c r="C7" s="22"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="22"/>
+      <c r="F7" s="22"/>
       <c r="G7" s="13"/>
       <c r="H7" s="14"/>
       <c r="I7" s="13"/>
@@ -812,12 +815,12 @@
       <c r="R7" s="14"/>
     </row>
     <row r="8" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
+      <c r="A8" s="22"/>
+      <c r="B8" s="22"/>
+      <c r="C8" s="22"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="22"/>
+      <c r="F8" s="22"/>
       <c r="G8" s="15"/>
       <c r="H8" s="16"/>
       <c r="I8" s="15"/>
@@ -832,473 +835,453 @@
       <c r="R8" s="16"/>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A9" s="4">
+      <c r="A9" s="10">
         <v>46094</v>
       </c>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3" t="s">
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="5" t="s">
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H9" s="7"/>
+      <c r="H9" s="3"/>
       <c r="I9" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="J9" s="6"/>
-      <c r="K9" s="6"/>
-      <c r="L9" s="6"/>
-      <c r="M9" s="6"/>
-      <c r="N9" s="6"/>
-      <c r="O9" s="6"/>
-      <c r="P9" s="6"/>
-      <c r="Q9" s="6"/>
-      <c r="R9" s="7"/>
+      <c r="J9" s="2"/>
+      <c r="K9" s="2"/>
+      <c r="L9" s="2"/>
+      <c r="M9" s="2"/>
+      <c r="N9" s="2"/>
+      <c r="O9" s="2"/>
+      <c r="P9" s="2"/>
+      <c r="Q9" s="2"/>
+      <c r="R9" s="3"/>
     </row>
     <row r="10" spans="1:18" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="8"/>
-      <c r="H10" s="10"/>
-      <c r="I10" s="8"/>
-      <c r="J10" s="9"/>
-      <c r="K10" s="9"/>
-      <c r="L10" s="9"/>
-      <c r="M10" s="9"/>
-      <c r="N10" s="9"/>
-      <c r="O10" s="9"/>
-      <c r="P10" s="9"/>
-      <c r="Q10" s="9"/>
-      <c r="R10" s="10"/>
+      <c r="A10" s="7"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="4"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="4"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5"/>
+      <c r="M10" s="5"/>
+      <c r="N10" s="5"/>
+      <c r="O10" s="5"/>
+      <c r="P10" s="5"/>
+      <c r="Q10" s="5"/>
+      <c r="R10" s="6"/>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A11" s="4">
+      <c r="A11" s="10">
         <v>46098</v>
       </c>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3" t="s">
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="5" t="s">
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H11" s="7"/>
-      <c r="I11" s="5" t="s">
+      <c r="H11" s="3"/>
+      <c r="I11" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J11" s="6"/>
-      <c r="K11" s="6"/>
-      <c r="L11" s="6"/>
-      <c r="M11" s="6"/>
-      <c r="N11" s="6"/>
-      <c r="O11" s="6"/>
-      <c r="P11" s="6"/>
-      <c r="Q11" s="6"/>
-      <c r="R11" s="7"/>
+      <c r="J11" s="2"/>
+      <c r="K11" s="2"/>
+      <c r="L11" s="2"/>
+      <c r="M11" s="2"/>
+      <c r="N11" s="2"/>
+      <c r="O11" s="2"/>
+      <c r="P11" s="2"/>
+      <c r="Q11" s="2"/>
+      <c r="R11" s="3"/>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="8"/>
-      <c r="H12" s="10"/>
-      <c r="I12" s="8"/>
-      <c r="J12" s="9"/>
-      <c r="K12" s="9"/>
-      <c r="L12" s="9"/>
-      <c r="M12" s="9"/>
-      <c r="N12" s="9"/>
-      <c r="O12" s="9"/>
-      <c r="P12" s="9"/>
-      <c r="Q12" s="9"/>
-      <c r="R12" s="10"/>
+      <c r="A12" s="7"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="4"/>
+      <c r="H12" s="6"/>
+      <c r="I12" s="4"/>
+      <c r="J12" s="5"/>
+      <c r="K12" s="5"/>
+      <c r="L12" s="5"/>
+      <c r="M12" s="5"/>
+      <c r="N12" s="5"/>
+      <c r="O12" s="5"/>
+      <c r="P12" s="5"/>
+      <c r="Q12" s="5"/>
+      <c r="R12" s="6"/>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A13" s="4">
+      <c r="A13" s="10">
         <v>46104</v>
       </c>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3" t="s">
+      <c r="B13" s="7"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="5" t="s">
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="H13" s="7"/>
-      <c r="I13" s="5"/>
-      <c r="J13" s="6"/>
-      <c r="K13" s="6"/>
-      <c r="L13" s="6"/>
-      <c r="M13" s="6"/>
-      <c r="N13" s="6"/>
-      <c r="O13" s="6"/>
-      <c r="P13" s="6"/>
-      <c r="Q13" s="6"/>
-      <c r="R13" s="7"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="1"/>
+      <c r="J13" s="2"/>
+      <c r="K13" s="2"/>
+      <c r="L13" s="2"/>
+      <c r="M13" s="2"/>
+      <c r="N13" s="2"/>
+      <c r="O13" s="2"/>
+      <c r="P13" s="2"/>
+      <c r="Q13" s="2"/>
+      <c r="R13" s="3"/>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="8"/>
-      <c r="H14" s="10"/>
-      <c r="I14" s="8"/>
-      <c r="J14" s="9"/>
-      <c r="K14" s="9"/>
-      <c r="L14" s="9"/>
-      <c r="M14" s="9"/>
-      <c r="N14" s="9"/>
-      <c r="O14" s="9"/>
-      <c r="P14" s="9"/>
-      <c r="Q14" s="9"/>
-      <c r="R14" s="10"/>
+      <c r="A14" s="7"/>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="4"/>
+      <c r="H14" s="6"/>
+      <c r="I14" s="4"/>
+      <c r="J14" s="5"/>
+      <c r="K14" s="5"/>
+      <c r="L14" s="5"/>
+      <c r="M14" s="5"/>
+      <c r="N14" s="5"/>
+      <c r="O14" s="5"/>
+      <c r="P14" s="5"/>
+      <c r="Q14" s="5"/>
+      <c r="R14" s="6"/>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="5" t="s">
+      <c r="A15" s="7"/>
+      <c r="B15" s="7"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H15" s="7"/>
-      <c r="I15" s="5"/>
-      <c r="J15" s="6"/>
-      <c r="K15" s="6"/>
-      <c r="L15" s="6"/>
-      <c r="M15" s="6"/>
-      <c r="N15" s="6"/>
-      <c r="O15" s="6"/>
-      <c r="P15" s="6"/>
-      <c r="Q15" s="6"/>
-      <c r="R15" s="7"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="1"/>
+      <c r="J15" s="2"/>
+      <c r="K15" s="2"/>
+      <c r="L15" s="2"/>
+      <c r="M15" s="2"/>
+      <c r="N15" s="2"/>
+      <c r="O15" s="2"/>
+      <c r="P15" s="2"/>
+      <c r="Q15" s="2"/>
+      <c r="R15" s="3"/>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A16" s="3"/>
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="10"/>
-      <c r="I16" s="8"/>
-      <c r="J16" s="9"/>
-      <c r="K16" s="9"/>
-      <c r="L16" s="9"/>
-      <c r="M16" s="9"/>
-      <c r="N16" s="9"/>
-      <c r="O16" s="9"/>
-      <c r="P16" s="9"/>
-      <c r="Q16" s="9"/>
-      <c r="R16" s="10"/>
+      <c r="A16" s="7"/>
+      <c r="B16" s="7"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
+      <c r="G16" s="4"/>
+      <c r="H16" s="6"/>
+      <c r="I16" s="4"/>
+      <c r="J16" s="5"/>
+      <c r="K16" s="5"/>
+      <c r="L16" s="5"/>
+      <c r="M16" s="5"/>
+      <c r="N16" s="5"/>
+      <c r="O16" s="5"/>
+      <c r="P16" s="5"/>
+      <c r="Q16" s="5"/>
+      <c r="R16" s="6"/>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="5" t="s">
+      <c r="A17" s="7"/>
+      <c r="B17" s="7"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="H17" s="7"/>
-      <c r="I17" s="5"/>
-      <c r="J17" s="6"/>
-      <c r="K17" s="6"/>
-      <c r="L17" s="6"/>
-      <c r="M17" s="6"/>
-      <c r="N17" s="6"/>
-      <c r="O17" s="6"/>
-      <c r="P17" s="6"/>
-      <c r="Q17" s="6"/>
-      <c r="R17" s="7"/>
+      <c r="H17" s="3"/>
+      <c r="I17" s="1"/>
+      <c r="J17" s="2"/>
+      <c r="K17" s="2"/>
+      <c r="L17" s="2"/>
+      <c r="M17" s="2"/>
+      <c r="N17" s="2"/>
+      <c r="O17" s="2"/>
+      <c r="P17" s="2"/>
+      <c r="Q17" s="2"/>
+      <c r="R17" s="3"/>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A18" s="3"/>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="10"/>
-      <c r="I18" s="8"/>
-      <c r="J18" s="9"/>
-      <c r="K18" s="9"/>
-      <c r="L18" s="9"/>
-      <c r="M18" s="9"/>
-      <c r="N18" s="9"/>
-      <c r="O18" s="9"/>
-      <c r="P18" s="9"/>
-      <c r="Q18" s="9"/>
-      <c r="R18" s="10"/>
+      <c r="A18" s="7"/>
+      <c r="B18" s="7"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="4"/>
+      <c r="H18" s="6"/>
+      <c r="I18" s="4"/>
+      <c r="J18" s="5"/>
+      <c r="K18" s="5"/>
+      <c r="L18" s="5"/>
+      <c r="M18" s="5"/>
+      <c r="N18" s="5"/>
+      <c r="O18" s="5"/>
+      <c r="P18" s="5"/>
+      <c r="Q18" s="5"/>
+      <c r="R18" s="6"/>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="5" t="s">
+      <c r="A19" s="7"/>
+      <c r="B19" s="7"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H19" s="7"/>
-      <c r="I19" s="5"/>
-      <c r="J19" s="6"/>
-      <c r="K19" s="6"/>
-      <c r="L19" s="6"/>
-      <c r="M19" s="6"/>
-      <c r="N19" s="6"/>
-      <c r="O19" s="6"/>
-      <c r="P19" s="6"/>
-      <c r="Q19" s="6"/>
-      <c r="R19" s="7"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="1"/>
+      <c r="J19" s="2"/>
+      <c r="K19" s="2"/>
+      <c r="L19" s="2"/>
+      <c r="M19" s="2"/>
+      <c r="N19" s="2"/>
+      <c r="O19" s="2"/>
+      <c r="P19" s="2"/>
+      <c r="Q19" s="2"/>
+      <c r="R19" s="3"/>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
-      <c r="G20" s="8"/>
-      <c r="H20" s="10"/>
-      <c r="I20" s="8"/>
-      <c r="J20" s="9"/>
-      <c r="K20" s="9"/>
-      <c r="L20" s="9"/>
-      <c r="M20" s="9"/>
-      <c r="N20" s="9"/>
-      <c r="O20" s="9"/>
-      <c r="P20" s="9"/>
-      <c r="Q20" s="9"/>
-      <c r="R20" s="10"/>
+      <c r="A20" s="7"/>
+      <c r="B20" s="7"/>
+      <c r="C20" s="7"/>
+      <c r="D20" s="7"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="7"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="6"/>
+      <c r="I20" s="4"/>
+      <c r="J20" s="5"/>
+      <c r="K20" s="5"/>
+      <c r="L20" s="5"/>
+      <c r="M20" s="5"/>
+      <c r="N20" s="5"/>
+      <c r="O20" s="5"/>
+      <c r="P20" s="5"/>
+      <c r="Q20" s="5"/>
+      <c r="R20" s="6"/>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A21" s="3"/>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
-      <c r="F21" s="3"/>
-      <c r="G21" s="3" t="s">
+      <c r="A21" s="7"/>
+      <c r="B21" s="7"/>
+      <c r="C21" s="7"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="H21" s="3"/>
-      <c r="I21" s="3"/>
-      <c r="J21" s="3"/>
-      <c r="K21" s="3"/>
-      <c r="L21" s="3"/>
-      <c r="M21" s="3"/>
-      <c r="N21" s="3"/>
-      <c r="O21" s="3"/>
-      <c r="P21" s="3"/>
-      <c r="Q21" s="3"/>
-      <c r="R21" s="3"/>
+      <c r="H21" s="7"/>
+      <c r="I21" s="7"/>
+      <c r="J21" s="7"/>
+      <c r="K21" s="7"/>
+      <c r="L21" s="7"/>
+      <c r="M21" s="7"/>
+      <c r="N21" s="7"/>
+      <c r="O21" s="7"/>
+      <c r="P21" s="7"/>
+      <c r="Q21" s="7"/>
+      <c r="R21" s="7"/>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A22" s="3"/>
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
-      <c r="F22" s="3"/>
-      <c r="G22" s="3"/>
-      <c r="H22" s="3"/>
-      <c r="I22" s="3"/>
-      <c r="J22" s="3"/>
-      <c r="K22" s="3"/>
-      <c r="L22" s="3"/>
-      <c r="M22" s="3"/>
-      <c r="N22" s="3"/>
-      <c r="O22" s="3"/>
-      <c r="P22" s="3"/>
-      <c r="Q22" s="3"/>
-      <c r="R22" s="3"/>
+      <c r="A22" s="7"/>
+      <c r="B22" s="7"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="7"/>
+      <c r="G22" s="7"/>
+      <c r="H22" s="7"/>
+      <c r="I22" s="7"/>
+      <c r="J22" s="7"/>
+      <c r="K22" s="7"/>
+      <c r="L22" s="7"/>
+      <c r="M22" s="7"/>
+      <c r="N22" s="7"/>
+      <c r="O22" s="7"/>
+      <c r="P22" s="7"/>
+      <c r="Q22" s="7"/>
+      <c r="R22" s="7"/>
     </row>
     <row r="23" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="22"/>
-      <c r="B23" s="22"/>
-      <c r="C23" s="22"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="22"/>
-      <c r="F23" s="22"/>
-      <c r="G23" s="22"/>
-      <c r="H23" s="22"/>
-      <c r="I23" s="22"/>
-      <c r="J23" s="22"/>
-      <c r="K23" s="22"/>
-      <c r="L23" s="22"/>
-      <c r="M23" s="22"/>
-      <c r="N23" s="22"/>
-      <c r="O23" s="22"/>
-      <c r="P23" s="22"/>
-      <c r="Q23" s="22"/>
-      <c r="R23" s="22"/>
+      <c r="A23" s="8"/>
+      <c r="B23" s="8"/>
+      <c r="C23" s="8"/>
+      <c r="D23" s="8"/>
+      <c r="E23" s="8"/>
+      <c r="F23" s="8"/>
+      <c r="G23" s="8"/>
+      <c r="H23" s="8"/>
+      <c r="I23" s="8"/>
+      <c r="J23" s="8"/>
+      <c r="K23" s="8"/>
+      <c r="L23" s="8"/>
+      <c r="M23" s="8"/>
+      <c r="N23" s="8"/>
+      <c r="O23" s="8"/>
+      <c r="P23" s="8"/>
+      <c r="Q23" s="8"/>
+      <c r="R23" s="8"/>
     </row>
     <row r="24" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="23"/>
-      <c r="B24" s="23"/>
-      <c r="C24" s="23"/>
-      <c r="D24" s="23"/>
-      <c r="E24" s="23"/>
-      <c r="F24" s="23"/>
-      <c r="G24" s="23"/>
-      <c r="H24" s="23"/>
-      <c r="I24" s="23"/>
-      <c r="J24" s="23"/>
-      <c r="K24" s="23"/>
-      <c r="L24" s="23"/>
-      <c r="M24" s="23"/>
-      <c r="N24" s="23"/>
-      <c r="O24" s="23"/>
-      <c r="P24" s="23"/>
-      <c r="Q24" s="23"/>
-      <c r="R24" s="23"/>
+      <c r="A24" s="9"/>
+      <c r="B24" s="9"/>
+      <c r="C24" s="9"/>
+      <c r="D24" s="9"/>
+      <c r="E24" s="9"/>
+      <c r="F24" s="9"/>
+      <c r="G24" s="9"/>
+      <c r="H24" s="9"/>
+      <c r="I24" s="9"/>
+      <c r="J24" s="9"/>
+      <c r="K24" s="9"/>
+      <c r="L24" s="9"/>
+      <c r="M24" s="9"/>
+      <c r="N24" s="9"/>
+      <c r="O24" s="9"/>
+      <c r="P24" s="9"/>
+      <c r="Q24" s="9"/>
+      <c r="R24" s="9"/>
     </row>
     <row r="25" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="4">
+      <c r="A25" s="10">
         <v>46095</v>
       </c>
-      <c r="B25" s="3"/>
-      <c r="C25" s="3"/>
-      <c r="D25" s="3" t="s">
+      <c r="B25" s="7"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="E25" s="3"/>
-      <c r="F25" s="3"/>
-      <c r="G25" s="3" t="s">
+      <c r="E25" s="7"/>
+      <c r="F25" s="7"/>
+      <c r="G25" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H25" s="3"/>
-      <c r="I25" s="3" t="s">
+      <c r="H25" s="7"/>
+      <c r="I25" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="J25" s="3"/>
-      <c r="K25" s="3"/>
-      <c r="L25" s="3"/>
-      <c r="M25" s="3"/>
-      <c r="N25" s="3"/>
-      <c r="O25" s="3"/>
-      <c r="P25" s="3"/>
-      <c r="Q25" s="3"/>
-      <c r="R25" s="3"/>
+      <c r="J25" s="7"/>
+      <c r="K25" s="7"/>
+      <c r="L25" s="7"/>
+      <c r="M25" s="7"/>
+      <c r="N25" s="7"/>
+      <c r="O25" s="7"/>
+      <c r="P25" s="7"/>
+      <c r="Q25" s="7"/>
+      <c r="R25" s="7"/>
     </row>
     <row r="26" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="3"/>
-      <c r="B26" s="3"/>
-      <c r="C26" s="3"/>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
-      <c r="G26" s="3"/>
-      <c r="H26" s="3"/>
-      <c r="I26" s="3"/>
-      <c r="J26" s="3"/>
-      <c r="K26" s="3"/>
-      <c r="L26" s="3"/>
-      <c r="M26" s="3"/>
-      <c r="N26" s="3"/>
-      <c r="O26" s="3"/>
-      <c r="P26" s="3"/>
-      <c r="Q26" s="3"/>
-      <c r="R26" s="3"/>
+      <c r="A26" s="7"/>
+      <c r="B26" s="7"/>
+      <c r="C26" s="7"/>
+      <c r="D26" s="7"/>
+      <c r="E26" s="7"/>
+      <c r="F26" s="7"/>
+      <c r="G26" s="7"/>
+      <c r="H26" s="7"/>
+      <c r="I26" s="7"/>
+      <c r="J26" s="7"/>
+      <c r="K26" s="7"/>
+      <c r="L26" s="7"/>
+      <c r="M26" s="7"/>
+      <c r="N26" s="7"/>
+      <c r="O26" s="7"/>
+      <c r="P26" s="7"/>
+      <c r="Q26" s="7"/>
+      <c r="R26" s="7"/>
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A27" s="21"/>
-      <c r="B27" s="21"/>
-      <c r="C27" s="21"/>
-      <c r="D27" s="21"/>
-      <c r="E27" s="21"/>
-      <c r="F27" s="21"/>
-      <c r="G27" s="3" t="s">
+      <c r="A27" s="10">
+        <v>46102</v>
+      </c>
+      <c r="B27" s="7"/>
+      <c r="C27" s="7"/>
+      <c r="D27" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="E27" s="7"/>
+      <c r="F27" s="7"/>
+      <c r="G27" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="H27" s="3"/>
-      <c r="I27" s="3"/>
-      <c r="J27" s="3"/>
-      <c r="K27" s="3"/>
-      <c r="L27" s="3"/>
-      <c r="M27" s="3"/>
-      <c r="N27" s="3"/>
-      <c r="O27" s="3"/>
-      <c r="P27" s="3"/>
-      <c r="Q27" s="3"/>
-      <c r="R27" s="3"/>
+      <c r="H27" s="7"/>
+      <c r="I27" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="J27" s="7"/>
+      <c r="K27" s="7"/>
+      <c r="L27" s="7"/>
+      <c r="M27" s="7"/>
+      <c r="N27" s="7"/>
+      <c r="O27" s="7"/>
+      <c r="P27" s="7"/>
+      <c r="Q27" s="7"/>
+      <c r="R27" s="7"/>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A28" s="21"/>
-      <c r="B28" s="21"/>
-      <c r="C28" s="21"/>
-      <c r="D28" s="21"/>
-      <c r="E28" s="21"/>
-      <c r="F28" s="21"/>
-      <c r="G28" s="3"/>
-      <c r="H28" s="3"/>
-      <c r="I28" s="3"/>
-      <c r="J28" s="3"/>
-      <c r="K28" s="3"/>
-      <c r="L28" s="3"/>
-      <c r="M28" s="3"/>
-      <c r="N28" s="3"/>
-      <c r="O28" s="3"/>
-      <c r="P28" s="3"/>
-      <c r="Q28" s="3"/>
-      <c r="R28" s="3"/>
+      <c r="A28" s="7"/>
+      <c r="B28" s="7"/>
+      <c r="C28" s="7"/>
+      <c r="D28" s="7"/>
+      <c r="E28" s="7"/>
+      <c r="F28" s="7"/>
+      <c r="G28" s="7"/>
+      <c r="H28" s="7"/>
+      <c r="I28" s="7"/>
+      <c r="J28" s="7"/>
+      <c r="K28" s="7"/>
+      <c r="L28" s="7"/>
+      <c r="M28" s="7"/>
+      <c r="N28" s="7"/>
+      <c r="O28" s="7"/>
+      <c r="P28" s="7"/>
+      <c r="Q28" s="7"/>
+      <c r="R28" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="42">
-    <mergeCell ref="I15:R16"/>
-    <mergeCell ref="G25:H26"/>
-    <mergeCell ref="G27:H28"/>
-    <mergeCell ref="A23:R24"/>
-    <mergeCell ref="I25:R26"/>
-    <mergeCell ref="I27:R28"/>
-    <mergeCell ref="D25:F26"/>
-    <mergeCell ref="D27:F28"/>
-    <mergeCell ref="A25:C26"/>
-    <mergeCell ref="A27:C28"/>
-    <mergeCell ref="A17:C18"/>
-    <mergeCell ref="I17:R18"/>
-    <mergeCell ref="I19:R20"/>
-    <mergeCell ref="I21:R22"/>
-    <mergeCell ref="G3:H8"/>
-    <mergeCell ref="G9:H10"/>
-    <mergeCell ref="G11:H12"/>
-    <mergeCell ref="G15:H16"/>
-    <mergeCell ref="G13:H14"/>
-    <mergeCell ref="G17:H18"/>
-    <mergeCell ref="G19:H20"/>
-    <mergeCell ref="G21:H22"/>
-    <mergeCell ref="I3:R8"/>
-    <mergeCell ref="I9:R10"/>
-    <mergeCell ref="I11:R12"/>
-    <mergeCell ref="I13:R14"/>
     <mergeCell ref="A1:R2"/>
     <mergeCell ref="A3:C8"/>
     <mergeCell ref="D3:F8"/>
@@ -1315,6 +1298,32 @@
     <mergeCell ref="A11:C12"/>
     <mergeCell ref="A13:C14"/>
     <mergeCell ref="A15:C16"/>
+    <mergeCell ref="G21:H22"/>
+    <mergeCell ref="I3:R8"/>
+    <mergeCell ref="I9:R10"/>
+    <mergeCell ref="I11:R12"/>
+    <mergeCell ref="I13:R14"/>
+    <mergeCell ref="G3:H8"/>
+    <mergeCell ref="G9:H10"/>
+    <mergeCell ref="G11:H12"/>
+    <mergeCell ref="G15:H16"/>
+    <mergeCell ref="G13:H14"/>
+    <mergeCell ref="I15:R16"/>
+    <mergeCell ref="G25:H26"/>
+    <mergeCell ref="G27:H28"/>
+    <mergeCell ref="A23:R24"/>
+    <mergeCell ref="I25:R26"/>
+    <mergeCell ref="I27:R28"/>
+    <mergeCell ref="D25:F26"/>
+    <mergeCell ref="D27:F28"/>
+    <mergeCell ref="A25:C26"/>
+    <mergeCell ref="A27:C28"/>
+    <mergeCell ref="A17:C18"/>
+    <mergeCell ref="I17:R18"/>
+    <mergeCell ref="I19:R20"/>
+    <mergeCell ref="I21:R22"/>
+    <mergeCell ref="G17:H18"/>
+    <mergeCell ref="G19:H20"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>